<commit_message>
checkpoint before agent handoff
</commit_message>
<xml_diff>
--- a/00 - definicion de landscape tsi/Relaciones.xlsx
+++ b/00 - definicion de landscape tsi/Relaciones.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JLAU\landscape tsi\00 - definicion de landscape tsi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4758A502-BCC1-4EE9-B3E6-8E8DFDBE3027}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60CB868F-A58D-490B-A141-AAAE507BF615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="56">
   <si>
     <t>Nombre en el modelado</t>
   </si>
@@ -165,9 +165,6 @@
     <t>EstadoFaseAdopcion</t>
   </si>
   <si>
-    <t>Postura Roadmap,</t>
-  </si>
-  <si>
     <t>TMPosturaRoadmap</t>
   </si>
   <si>
@@ -187,6 +184,15 @@
   </si>
   <si>
     <t>TModalidadLaboral</t>
+  </si>
+  <si>
+    <t>ROL Owner</t>
+  </si>
+  <si>
+    <t>Arquitecto de Seguridad Corporativo</t>
+  </si>
+  <si>
+    <t>Postura Roadmap</t>
   </si>
 </sst>
 </file>
@@ -224,7 +230,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -232,19 +238,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -527,315 +555,379 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:E20"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="6" width="27.7109375" customWidth="1"/>
+    <col min="1" max="1" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="27.7109375" customWidth="1"/>
+    <col min="4" max="5" width="27.7109375" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="47.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="F1" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="D2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="F2" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="D3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="F3" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="D4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="F4" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="D5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="D6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="F6" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="C7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>45</v>
+      </c>
       <c r="C8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E14" s="1"/>
+      <c r="F14" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="1"/>
+      <c r="F15" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" s="1"/>
+      <c r="F16" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" s="1"/>
+      <c r="F17" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>8</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>9</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>10</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>11</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>12</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>13</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="B19" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>14</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E16" s="2" t="s">
+      <c r="E19" s="3" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>15</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>16</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>17</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>18</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>6</v>
+      <c r="F19" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>